<commit_message>
feat(notebooklm & docs): Nap 11 tai lieu vao Bo nao NotebookLM UNIGO, cap nhat TKB giao vien, Ke hoach Van Mieu va Slide Tuan 04
</commit_message>
<xml_diff>
--- a/Hệ thống mẫu văn bản/Nguyên đã làm/Thời khóa biểu/Thời khóa biểu - Đậu Đình Nguyên.xlsx
+++ b/Hệ thống mẫu văn bản/Nguyên đã làm/Thời khóa biểu/Thời khóa biểu - Đậu Đình Nguyên.xlsx
@@ -323,16 +323,16 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -846,8 +846,8 @@
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>🤖 Robotics
-(3C1)</t>
+          <t>💻 Tin học
+(2A1)</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,12 @@
 (1A1)</t>
         </is>
       </c>
-      <c r="H8" s="18" t="n"/>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>🤖 Robotics
+(3C1)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
@@ -913,7 +918,7 @@
       </c>
       <c r="F9" s="14" t="n"/>
       <c r="G9" s="14" t="n"/>
-      <c r="H9" s="18" t="n"/>
+      <c r="H9" s="19" t="n"/>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
@@ -955,7 +960,7 @@
 (2C1)</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="H10" s="16" t="inlineStr">
         <is>
           <t>💻 Tin học
 (6A1)</t>
@@ -978,7 +983,7 @@
       <c r="E11" s="14" t="n"/>
       <c r="F11" s="14" t="n"/>
       <c r="G11" s="14" t="n"/>
-      <c r="H11" s="16" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>🤖 Robotics
 (6A1)</t>
@@ -1016,12 +1021,7 @@
         </is>
       </c>
       <c r="D13" s="14" t="n"/>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>💻 Tin học
-(2A1)</t>
-        </is>
-      </c>
+      <c r="E13" s="14" t="n"/>
       <c r="F13" s="14" t="n"/>
       <c r="G13" s="15" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
 (3A1)</t>
         </is>
       </c>
-      <c r="H13" s="19" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>💻 Tin học
 (8A1)</t>
@@ -1061,7 +1061,7 @@
 (TTH 1)</t>
         </is>
       </c>
-      <c r="H14" s="16" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>🤖 Robotics
 (8A1)</t>
@@ -1108,7 +1108,7 @@
 (TTH2)</t>
         </is>
       </c>
-      <c r="H15" s="18" t="n"/>
+      <c r="H15" s="19" t="n"/>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
@@ -1145,7 +1145,7 @@
 (1C1)</t>
         </is>
       </c>
-      <c r="H16" s="18" t="n"/>
+      <c r="H16" s="19" t="n"/>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="20" t="inlineStr">

</xml_diff>